<commit_message>
Add Notes tab and a flat all-fixtures CSV
The flat CSV is what gets uploaded to Drive: passing it as text avoids the
base64 round-trip that xlsx upload requires, which is where the earlier
Sunday-tab data loss came from.
</commit_message>
<xml_diff>
--- a/english-open-2026/english-open-2026-full.xlsx
+++ b/english-open-2026/english-open-2026-full.xlsx
@@ -22,6 +22,7 @@
     <sheet name="Sophie Maitland" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="Jack Adams" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="Sonja Talbot" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Notes" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -202,7 +203,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -362,6 +363,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3846,6 +3853,114 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="96" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Worth reading once before the weekend</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="54" t="inlineStr">
+        <is>
+          <t>Where this came from</t>
+        </is>
+      </c>
+      <c r="B4" s="55" t="inlineStr">
+        <is>
+          <t>Transcribed from the tournament's Schedule &amp; Results screens on PickleBook, filtered to each player in turn. 64 unique matches across the ten of us.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="54" t="inlineStr">
+        <is>
+          <t>How it was checked</t>
+        </is>
+      </c>
+      <c r="B5" s="55" t="inlineStr">
+        <is>
+          <t>Each player's match count reconciles exactly against the entry total PickleBook showed on their filtered view. No player was double-booked and no two matches sit close together in different zones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="54" t="inlineStr">
+        <is>
+          <t>Names</t>
+        </is>
+      </c>
+      <c r="B6" s="55" t="inlineStr">
+        <is>
+          <t>As registered on PickleBook — Will Cheeseman (not William), and Tracey-Anne under Greenhow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="54" t="inlineStr">
+        <is>
+          <t>Withdrawal</t>
+        </is>
+      </c>
+      <c r="B7" s="55" t="inlineStr">
+        <is>
+          <t>Match #15652, Sunday 14:40 on Court 47 — Holly and James's opponents are struck out on PickleBook and marked withdrawn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="54" t="inlineStr">
+        <is>
+          <t>Times</t>
+        </is>
+      </c>
+      <c r="B8" s="55" t="inlineStr">
+        <is>
+          <t>Scheduled starts only. Tournament days drift; the live board at the venue wins.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="54" t="inlineStr">
+        <is>
+          <t>One thing unverified</t>
+        </is>
+      </c>
+      <c r="B9" s="55" t="inlineStr">
+        <is>
+          <t>Every source view had the Status filter set to 'A'. If that is a status code rather than 'All', fixtures in other states would not appear here.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>